<commit_message>
Updated all changes n modules
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hema.ananthan\eclipse-workspace\com.ggproduct.automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A378E913-5003-45BF-B102-3A2AA37EDBEF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E642EB-DED5-4BE0-80BF-FF49471EDABC}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" activeTab="3" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>NewBudgetPeriodEndDate__c</t>
+  </si>
+  <si>
+    <t>InternalAmendmentType__c</t>
   </si>
 </sst>
 </file>
@@ -494,7 +497,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
@@ -524,6 +527,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Merged PR 2024: Merge applicationintake-refactoring to master
Refactoring
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E642EB-DED5-4BE0-80BF-FF49471EDABC}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1064210-F6FD-40BA-BB43-AEFCEFC4B8C8}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8964" activeTab="2" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="27">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>None</t>
-  </si>
-  <si>
-    <t>AmendmentType__c</t>
   </si>
   <si>
     <t>Scope of Work Change</t>
@@ -497,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -508,10 +505,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -519,10 +516,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -554,87 +551,87 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
         <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>18</v>
-      </c>
-      <c r="C7" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
         <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9">
         <v>12345</v>
@@ -642,13 +639,13 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
         <v>23</v>
-      </c>
-      <c r="C10" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -681,10 +678,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -692,10 +689,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -703,10 +700,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -736,10 +733,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C2">
         <v>400</v>

</xml_diff>

<commit_message>
Merged PR 2836: Merge mfixes to master
Added new test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,22 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1064210-F6FD-40BA-BB43-AEFCEFC4B8C8}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4011367-C0BF-4574-8C28-1D80CC479C57}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8964" activeTab="2" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="2" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
     <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId2"/>
     <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId3"/>
     <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId4"/>
+    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId5"/>
+    <sheet name="GrantCreation" sheetId="6" r:id="rId6"/>
+    <sheet name="GrantEdition" sheetId="7" r:id="rId7"/>
+    <sheet name="Edition_Standalone" sheetId="8" r:id="rId8"/>
+    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId9"/>
+    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="71">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -114,19 +120,163 @@
   </si>
   <si>
     <t>InternalAmendmentType__c</t>
+  </si>
+  <si>
+    <t>fieldPurposeRTA__c</t>
+  </si>
+  <si>
+    <t>fieldImpact__c</t>
+  </si>
+  <si>
+    <t>Funding Change</t>
+  </si>
+  <si>
+    <t>ProjectTitle__c</t>
+  </si>
+  <si>
+    <t>GrantAbbreviation__c</t>
+  </si>
+  <si>
+    <t>GA</t>
+  </si>
+  <si>
+    <t>ProjectPeriodStartDate__c</t>
+  </si>
+  <si>
+    <t>ProjectPeriodEndDate__c</t>
+  </si>
+  <si>
+    <t>BudgetCategoryPackage__c</t>
+  </si>
+  <si>
+    <t>Construction</t>
+  </si>
+  <si>
+    <t>fieldInternalOrganization__c</t>
+  </si>
+  <si>
+    <t>SAN DIEGO ELECTRICAL TRAINING TRUST</t>
+  </si>
+  <si>
+    <t>Program__c</t>
+  </si>
+  <si>
+    <t>Automation Permanent Internal Program</t>
+  </si>
+  <si>
+    <t>ExternalOrganization__c</t>
+  </si>
+  <si>
+    <t>Test Automation Organization</t>
+  </si>
+  <si>
+    <t>IsMatchRequired__c</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>LaverageAllowed__c</t>
+  </si>
+  <si>
+    <t>IsProgramIncomeAnticipated__c</t>
+  </si>
+  <si>
+    <t>IsAdvancePermitted__c</t>
+  </si>
+  <si>
+    <t>IsBuildUpFunctionality__c</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>IsGoalsRequired__c</t>
+  </si>
+  <si>
+    <t>KPIsRequired__c</t>
+  </si>
+  <si>
+    <t>AreExpensesBuildIUpLevel__c</t>
+  </si>
+  <si>
+    <t>RiskAssessmentRequired__c</t>
+  </si>
+  <si>
+    <t>WBSRequired__c</t>
+  </si>
+  <si>
+    <t>FocusAreaRequired__c</t>
+  </si>
+  <si>
+    <t>GrantAwardDescription__c</t>
+  </si>
+  <si>
+    <t>Automation Test Description</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>BudgetPeriodEndDate__c</t>
+  </si>
+  <si>
+    <t>SubmissionTitle__c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation Payment Request </t>
+  </si>
+  <si>
+    <t>Frequency__c</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>ScheduleBase__c</t>
+  </si>
+  <si>
+    <t>Reporting Period</t>
+  </si>
+  <si>
+    <t>Description__c</t>
+  </si>
+  <si>
+    <t>CalReportingStartDate__c</t>
+  </si>
+  <si>
+    <t>CalReportingEndDate__c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation Progress Report </t>
+  </si>
+  <si>
+    <t>Automation Execution Award for Amendment Request</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF222222"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -149,13 +299,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -472,13 +626,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236FB0C8-BA27-46AC-83FF-CF70FBE95475}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -489,7 +643,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -500,7 +654,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -511,7 +665,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -528,17 +682,108 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3C3D45-7E71-472A-AB14-3D5373D782BA}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -549,7 +794,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -560,7 +805,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -571,7 +816,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -582,7 +827,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -593,7 +838,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -604,7 +849,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -615,7 +860,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -626,7 +871,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -637,7 +882,7 @@
         <v>12345</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -656,13 +901,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -673,7 +918,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -684,7 +929,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -695,7 +940,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -714,13 +959,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -731,7 +976,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -746,4 +991,460 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged PR 2889: Merge mfixes to master
Added new test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4011367-C0BF-4574-8C28-1D80CC479C57}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07FCA330-6883-4624-A771-6D3188CB41A1}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="2" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="3" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="72">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -252,6 +252,9 @@
   </si>
   <si>
     <t>Automation Execution Award for Amendment Request</t>
+  </si>
+  <si>
+    <t>fieldBudgetPeriodComments__c</t>
   </si>
 </sst>
 </file>
@@ -958,7 +961,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
@@ -984,7 +987,18 @@
         <v>25</v>
       </c>
       <c r="C2">
-        <v>400</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merged PR 2907: Merge mfixes to master
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07FCA330-6883-4624-A771-6D3188CB41A1}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F5D762-23FA-4AC4-9A85-5AE4AAE6F6E2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="3" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
@@ -17,12 +17,13 @@
     <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId2"/>
     <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId3"/>
     <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId4"/>
-    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId5"/>
-    <sheet name="GrantCreation" sheetId="6" r:id="rId6"/>
-    <sheet name="GrantEdition" sheetId="7" r:id="rId7"/>
-    <sheet name="Edition_Standalone" sheetId="8" r:id="rId8"/>
-    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId9"/>
-    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId10"/>
+    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId5"/>
+    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId6"/>
+    <sheet name="GrantCreation" sheetId="6" r:id="rId7"/>
+    <sheet name="GrantEdition" sheetId="7" r:id="rId8"/>
+    <sheet name="Edition_Standalone" sheetId="8" r:id="rId9"/>
+    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId10"/>
+    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="77">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -255,6 +256,21 @@
   </si>
   <si>
     <t>fieldBudgetPeriodComments__c</t>
+  </si>
+  <si>
+    <t>Financials</t>
+  </si>
+  <si>
+    <t>TermsAgreement__c</t>
+  </si>
+  <si>
+    <t>I Agree</t>
+  </si>
+  <si>
+    <t>ReceiptsUploaded__c</t>
+  </si>
+  <si>
+    <t>Checked</t>
   </si>
 </sst>
 </file>
@@ -686,6 +702,97 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -987,7 +1094,7 @@
         <v>25</v>
       </c>
       <c r="C2">
-        <v>30</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1008,6 +1115,53 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1066,7 +1220,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1179,7 +1333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1325,7 +1479,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1370,95 +1524,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7">
-        <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged PR 2929: Merge Deepika_prod to master
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F5D762-23FA-4AC4-9A85-5AE4AAE6F6E2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{619D12A6-FA9A-4DA6-805C-D523B0CE21D5}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="3" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="75">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -121,12 +121,6 @@
   </si>
   <si>
     <t>InternalAmendmentType__c</t>
-  </si>
-  <si>
-    <t>fieldPurposeRTA__c</t>
-  </si>
-  <si>
-    <t>fieldImpact__c</t>
   </si>
   <si>
     <t>Funding Change</t>
@@ -645,13 +639,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236FB0C8-BA27-46AC-83FF-CF70FBE95475}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -662,7 +656,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -673,7 +667,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -684,7 +678,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -704,13 +698,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -721,67 +715,67 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>60</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>62</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
         <v>64</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>67</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C7">
         <v>3650</v>
@@ -795,13 +789,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -812,67 +806,67 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>60</v>
       </c>
-      <c r="C2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>62</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
         <v>64</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>67</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C7">
         <v>3650</v>
@@ -886,14 +880,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3C3D45-7E71-472A-AB14-3D5373D782BA}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -904,7 +898,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -915,7 +909,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -926,7 +920,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -937,7 +931,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -948,7 +942,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -959,7 +953,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -970,7 +964,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -981,7 +975,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -992,7 +986,7 @@
         <v>12345</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1011,13 +1005,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1028,7 +1022,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1039,7 +1033,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1050,7 +1044,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1069,13 +1063,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1086,7 +1080,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1097,15 +1091,15 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1117,13 +1111,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1134,26 +1128,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" t="s">
         <v>72</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" t="s">
         <v>73</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" t="s">
-        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1164,13 +1158,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1181,34 +1175,34 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>27</v>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>28</v>
+      <c r="B4" t="s">
+        <v>7</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -1223,13 +1217,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1240,92 +1234,92 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>31</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>33</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C5">
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
         <v>37</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1336,13 +1330,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1353,125 +1347,125 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>43</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" t="s">
         <v>47</v>
       </c>
-      <c r="C5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>53</v>
       </c>
-      <c r="C10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>55</v>
-      </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1482,13 +1476,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1499,23 +1493,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>56</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B3" t="s">
-        <v>59</v>
       </c>
       <c r="C3">
         <v>3650</v>

</xml_diff>

<commit_message>
fixed failed test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{619D12A6-FA9A-4DA6-805C-D523B0CE21D5}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA28626-B98F-4FAD-AD06-96A4EEB9DD5D}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="5" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated old and added new TC
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Product Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA28626-B98F-4FAD-AD06-96A4EEB9DD5D}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DB6DA1-3C54-47C6-8C47-8F22B6CA794F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="5" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="10" activeTab="12" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,8 @@
     <sheet name="Edition_Standalone" sheetId="8" r:id="rId9"/>
     <sheet name="Payment Request Schedule" sheetId="9" r:id="rId10"/>
     <sheet name="Progress Report Schedule" sheetId="10" r:id="rId11"/>
+    <sheet name="Periodic Renewal" sheetId="12" r:id="rId12"/>
+    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="79">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -265,6 +267,18 @@
   </si>
   <si>
     <t>Checked</t>
+  </si>
+  <si>
+    <t>Periodic Renewal</t>
+  </si>
+  <si>
+    <t>ProposedBPStartDate__c</t>
+  </si>
+  <si>
+    <t>ProposedBudgetEndDate__c</t>
+  </si>
+  <si>
+    <t>fieldRequestedChangeInBudget__c</t>
   </si>
 </sst>
 </file>
@@ -639,13 +653,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236FB0C8-BA27-46AC-83FF-CF70FBE95475}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -656,7 +670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -667,7 +681,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -678,7 +692,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -698,13 +712,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -715,7 +729,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -726,7 +740,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -737,7 +751,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -748,7 +762,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -759,7 +773,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -770,7 +784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -789,13 +803,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -806,7 +820,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -817,7 +831,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -828,7 +842,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -839,7 +853,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -850,7 +864,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -861,7 +875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -874,20 +888,137 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF2024B-3855-4F21-818F-72BDEF018EB6}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6731B0-0A3A-4C99-9219-CD51FBCA919D}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4">
+        <v>1000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3C3D45-7E71-472A-AB14-3D5373D782BA}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -898,7 +1029,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -909,7 +1040,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -920,7 +1051,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -931,7 +1062,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -942,7 +1073,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -953,7 +1084,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -964,7 +1095,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -975,7 +1106,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -986,7 +1117,7 @@
         <v>12345</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1005,13 +1136,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1022,7 +1153,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1033,7 +1164,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1044,7 +1175,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1063,13 +1194,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1080,7 +1211,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1091,7 +1222,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1111,13 +1242,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1128,7 +1259,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>70</v>
       </c>
@@ -1139,7 +1270,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>70</v>
       </c>
@@ -1158,13 +1289,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1306,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1186,7 +1317,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1197,7 +1328,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1217,13 +1348,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1234,7 +1365,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1245,7 +1376,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1256,7 +1387,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1267,7 +1398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1278,7 +1409,7 @@
         <v>3650</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1289,7 +1420,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1300,7 +1431,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1311,7 +1442,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1330,13 +1461,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1347,7 +1478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1358,7 +1489,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1369,7 +1500,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1380,7 +1511,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1391,7 +1522,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1402,7 +1533,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1413,7 +1544,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1424,7 +1555,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1435,7 +1566,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1446,7 +1577,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1457,7 +1588,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1476,13 +1607,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1493,7 +1624,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1504,7 +1635,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
completed 10-11 test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -8,26 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A61B4E7-C495-476A-B285-5E6E8AF5BF2F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5C394D-86F4-4EDE-97C9-883B7F7732B9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="11" activeTab="13" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="8" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
-    <sheet name="Budget_Redirection" sheetId="15" r:id="rId2"/>
-    <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId3"/>
-    <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId4"/>
-    <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId5"/>
-    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId6"/>
-    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId7"/>
-    <sheet name="GrantCreation" sheetId="6" r:id="rId8"/>
-    <sheet name="GrantEdition" sheetId="7" r:id="rId9"/>
-    <sheet name="Edition_Standalone" sheetId="8" r:id="rId10"/>
-    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId11"/>
-    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId12"/>
-    <sheet name="Periodic Renewal" sheetId="12" r:id="rId13"/>
-    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId14"/>
-    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId15"/>
+    <sheet name="Subrecipient_SOW_creation" sheetId="17" r:id="rId2"/>
+    <sheet name="Budget_Redirection" sheetId="15" r:id="rId3"/>
+    <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId4"/>
+    <sheet name="Subrecipient_SOW_Edition" sheetId="18" r:id="rId5"/>
+    <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId6"/>
+    <sheet name="SubRecipientBPC_Creation" sheetId="19" r:id="rId7"/>
+    <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId8"/>
+    <sheet name="SubRecipientBPC_Edition" sheetId="20" r:id="rId9"/>
+    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId10"/>
+    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId11"/>
+    <sheet name="GrantCreation" sheetId="6" r:id="rId12"/>
+    <sheet name="GrantEdition" sheetId="7" r:id="rId13"/>
+    <sheet name="Edition_Standalone" sheetId="8" r:id="rId14"/>
+    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId15"/>
+    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId16"/>
+    <sheet name="Periodic Renewal" sheetId="12" r:id="rId17"/>
+    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId18"/>
+    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="86">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -284,13 +288,31 @@
   </si>
   <si>
     <t>Budget Redirection</t>
+  </si>
+  <si>
+    <t>fieldSubAmendmentType__c</t>
+  </si>
+  <si>
+    <t>fieldPurposeRTA__c</t>
+  </si>
+  <si>
+    <t>fieldImpact__c</t>
+  </si>
+  <si>
+    <t>fieldScopeofWorkChangeDescription__c</t>
+  </si>
+  <si>
+    <t>fieldCongressionaldistrict__c</t>
+  </si>
+  <si>
+    <t>fieldNewBudgetPeriodEndDate__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,6 +339,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF222222"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -338,7 +366,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -353,6 +381,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -725,6 +754,371 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="26.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.46484375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.1328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="30.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -771,7 +1165,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -862,7 +1256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -953,7 +1347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF2024B-3855-4F21-818F-72BDEF018EB6}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1011,7 +1405,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6731B0-0A3A-4C99-9219-CD51FBCA919D}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1059,7 +1453,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01F7F05-2D11-4E6A-A090-87D63AD5B8AF}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1118,6 +1512,66 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE5594E6-CDC4-4068-99A2-0F1E0C84230B}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="7.265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.59765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CED252CC-9A41-43A8-97A3-527BD171EFF4}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1177,7 +1631,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3C3D45-7E71-472A-AB14-3D5373D782BA}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1302,7 +1756,132 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B2B8548-7B25-4129-9EB7-BF1BA0DF00C4}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.9296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1360,7 +1939,66 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25797962-2CD8-4222-8F0C-F2737F68CB74}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.59765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1408,60 +2046,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F116B932-6CC5-49E6-907B-B1FB48B4CADD}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="26.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.46484375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
@@ -1477,295 +2069,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
+        <v>12</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2">
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+        <v>12</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.1328125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5">
-        <v>3650</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="30.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
completed 13 scenarios for Amendment request
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -8,30 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5C394D-86F4-4EDE-97C9-883B7F7732B9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05429BAD-1508-4A5D-AB63-DFD720BA9046}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="8" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="2" activeTab="4" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
     <sheet name="Subrecipient_SOW_creation" sheetId="17" r:id="rId2"/>
     <sheet name="Budget_Redirection" sheetId="15" r:id="rId3"/>
-    <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId4"/>
-    <sheet name="Subrecipient_SOW_Edition" sheetId="18" r:id="rId5"/>
-    <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId6"/>
-    <sheet name="SubRecipientBPC_Creation" sheetId="19" r:id="rId7"/>
-    <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId8"/>
-    <sheet name="SubRecipientBPC_Edition" sheetId="20" r:id="rId9"/>
-    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId10"/>
-    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId11"/>
-    <sheet name="GrantCreation" sheetId="6" r:id="rId12"/>
-    <sheet name="GrantEdition" sheetId="7" r:id="rId13"/>
-    <sheet name="Edition_Standalone" sheetId="8" r:id="rId14"/>
-    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId15"/>
-    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId16"/>
-    <sheet name="Periodic Renewal" sheetId="12" r:id="rId17"/>
-    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId18"/>
-    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId19"/>
+    <sheet name="Subrecipient_BRedirection" sheetId="21" r:id="rId4"/>
+    <sheet name="Subrecipient_KPC" sheetId="22" r:id="rId5"/>
+    <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId6"/>
+    <sheet name="Subrecipient_SOW_Edition" sheetId="18" r:id="rId7"/>
+    <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId8"/>
+    <sheet name="SubRecipientBPC_Creation" sheetId="19" r:id="rId9"/>
+    <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId10"/>
+    <sheet name="SubRecipientBPC_Edition" sheetId="20" r:id="rId11"/>
+    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId12"/>
+    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId13"/>
+    <sheet name="GrantCreation" sheetId="6" r:id="rId14"/>
+    <sheet name="GrantEdition" sheetId="7" r:id="rId15"/>
+    <sheet name="Edition_Standalone" sheetId="8" r:id="rId16"/>
+    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId17"/>
+    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId18"/>
+    <sheet name="Periodic Renewal" sheetId="12" r:id="rId19"/>
+    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId20"/>
+    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="87">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -306,6 +308,9 @@
   </si>
   <si>
     <t>fieldNewBudgetPeriodEndDate__c</t>
+  </si>
+  <si>
+    <t>Key Personnel Change</t>
   </si>
 </sst>
 </file>
@@ -754,6 +759,102 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="25.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.53125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F116B932-6CC5-49E6-907B-B1FB48B4CADD}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -800,7 +901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -859,7 +960,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -972,7 +1073,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1118,7 +1219,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1165,7 +1266,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1256,7 +1357,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1347,7 +1448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF2024B-3855-4F21-818F-72BDEF018EB6}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1376,112 +1477,6 @@
       </c>
       <c r="C2" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6731B0-0A3A-4C99-9219-CD51FBCA919D}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="30.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" s="5">
-        <v>4017</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C3">
-        <v>1000</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01F7F05-2D11-4E6A-A090-87D63AD5B8AF}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="24.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.59765625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -1571,6 +1566,112 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6731B0-0A3A-4C99-9219-CD51FBCA919D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="30.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="5">
+        <v>4017</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3">
+        <v>1000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01F7F05-2D11-4E6A-A090-87D63AD5B8AF}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="24.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.59765625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CED252CC-9A41-43A8-97A3-527BD171EFF4}">
   <dimension ref="A1:C4"/>
@@ -1632,6 +1733,123 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1C7C3E9-7A91-479E-8DB7-C5289494DF22}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="23.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F956442-5D32-41A9-9373-4CEFD36ACD4B}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3C3D45-7E71-472A-AB14-3D5373D782BA}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1756,7 +1974,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B2B8548-7B25-4129-9EB7-BF1BA0DF00C4}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1881,7 +2099,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1939,7 +2157,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25797962-2CD8-4222-8F0C-F2737F68CB74}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1996,100 +2214,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="25.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.53125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F116B932-6CC5-49E6-907B-B1FB48B4CADD}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="1" width="8.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
completed 10 scenario for Amendment Request
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05429BAD-1508-4A5D-AB63-DFD720BA9046}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771A19B6-4E6A-4E9B-8230-1166389000AC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="2" activeTab="4" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="9" activeTab="11" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -24,16 +24,17 @@
     <sheet name="SubRecipientBPC_Creation" sheetId="19" r:id="rId9"/>
     <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId10"/>
     <sheet name="SubRecipientBPC_Edition" sheetId="20" r:id="rId11"/>
-    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId12"/>
-    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId13"/>
-    <sheet name="GrantCreation" sheetId="6" r:id="rId14"/>
-    <sheet name="GrantEdition" sheetId="7" r:id="rId15"/>
-    <sheet name="Edition_Standalone" sheetId="8" r:id="rId16"/>
-    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId17"/>
-    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId18"/>
-    <sheet name="Periodic Renewal" sheetId="12" r:id="rId19"/>
-    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId20"/>
-    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId21"/>
+    <sheet name="SubRecipientCF_Creation" sheetId="23" r:id="rId12"/>
+    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId13"/>
+    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId14"/>
+    <sheet name="GrantCreation" sheetId="6" r:id="rId15"/>
+    <sheet name="GrantEdition" sheetId="7" r:id="rId16"/>
+    <sheet name="Edition_Standalone" sheetId="8" r:id="rId17"/>
+    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId18"/>
+    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId19"/>
+    <sheet name="Periodic Renewal" sheetId="12" r:id="rId20"/>
+    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId21"/>
+    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="88">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -311,6 +312,9 @@
   </si>
   <si>
     <t>Key Personnel Change</t>
+  </si>
+  <si>
+    <t>Carry Forward</t>
   </si>
 </sst>
 </file>
@@ -855,6 +859,64 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFB9B001-FDE9-4CB7-8749-6B43410AD625}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -901,7 +963,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -960,7 +1022,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1073,7 +1135,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1219,7 +1281,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1266,7 +1328,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1357,7 +1419,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1441,64 +1503,6 @@
       </c>
       <c r="C7">
         <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF2024B-3855-4F21-818F-72BDEF018EB6}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="26.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.46484375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1567,6 +1571,64 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF2024B-3855-4F21-818F-72BDEF018EB6}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="26.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.46484375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6731B0-0A3A-4C99-9219-CD51FBCA919D}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1614,7 +1676,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01F7F05-2D11-4E6A-A090-87D63AD5B8AF}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
Completed 13 test cases for UAT.
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771A19B6-4E6A-4E9B-8230-1166389000AC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96886475-6747-41B7-93AC-0A164D74A50C}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="9" activeTab="11" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" firstSheet="18" activeTab="19" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="89">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -315,6 +315,9 @@
   </si>
   <si>
     <t>Carry Forward</t>
+  </si>
+  <si>
+    <t>fieldInternalAmendmentType__c</t>
   </si>
 </sst>
 </file>
@@ -1595,7 +1598,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
         <v>75</v>
@@ -1606,7 +1609,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -1617,7 +1620,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
remove 1 Hold bug TC
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\product_automation_allocation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A140D94B-49D0-4F50-92B0-9063A267D266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6277D6-4BB6-4F22-B0F4-3B0178850DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="135" yWindow="390" windowWidth="20355" windowHeight="10920" firstSheet="21" activeTab="22" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="135" yWindow="390" windowWidth="20355" windowHeight="10920" firstSheet="24" activeTab="25" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="97">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -129,9 +129,6 @@
     <t>Congressionaldistrict__c</t>
   </si>
   <si>
-    <t>1st District</t>
-  </si>
-  <si>
     <t>Budget Period Change</t>
   </si>
   <si>
@@ -328,9 +325,6 @@
   </si>
   <si>
     <t>Automation Country</t>
-  </si>
-  <si>
-    <t>KA</t>
   </si>
   <si>
     <t>fieldState__c</t>
@@ -754,7 +748,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -785,7 +779,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -844,10 +838,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -855,7 +849,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -866,7 +860,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -903,10 +897,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -914,7 +908,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -925,7 +919,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -936,7 +930,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -972,7 +966,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C2">
         <v>70</v>
@@ -983,10 +977,10 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1021,7 +1015,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C2">
         <v>70</v>
@@ -1032,10 +1026,10 @@
         <v>12</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1068,10 +1062,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1079,7 +1073,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -1090,7 +1084,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -1123,24 +1117,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" t="s">
         <v>68</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>69</v>
-      </c>
-      <c r="C2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s">
         <v>71</v>
-      </c>
-      <c r="C3" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1173,10 +1167,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1232,10 +1226,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1243,10 +1237,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
         <v>27</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1254,7 +1248,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1265,7 +1259,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C5">
         <v>3650</v>
@@ -1276,10 +1270,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
         <v>31</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1287,10 +1281,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
         <v>33</v>
-      </c>
-      <c r="C7" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1298,10 +1292,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
         <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1309,10 +1303,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
         <v>37</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1345,10 +1339,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1356,10 +1350,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1367,10 +1361,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1378,10 +1372,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1389,10 +1383,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1400,10 +1394,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1411,10 +1405,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1422,10 +1416,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1433,10 +1427,10 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1444,10 +1438,10 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1455,10 +1449,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1491,18 +1485,18 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
         <v>52</v>
-      </c>
-      <c r="C2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" t="s">
         <v>54</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
       </c>
       <c r="C3">
         <v>3650</v>
@@ -1538,7 +1532,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -1549,10 +1543,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1607,10 +1601,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s">
         <v>56</v>
-      </c>
-      <c r="C2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1618,10 +1612,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
         <v>58</v>
-      </c>
-      <c r="C3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1629,10 +1623,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" t="s">
         <v>60</v>
-      </c>
-      <c r="C4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1640,10 +1634,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1651,7 +1645,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1662,7 +1656,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C7">
         <v>3650</v>
@@ -1698,10 +1692,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1709,10 +1703,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
         <v>58</v>
-      </c>
-      <c r="C3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1720,10 +1714,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" t="s">
         <v>60</v>
-      </c>
-      <c r="C4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1731,10 +1725,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1742,7 +1736,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1753,7 +1747,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C7">
         <v>3650</v>
@@ -1789,10 +1783,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1800,7 +1794,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -1811,7 +1805,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -1847,7 +1841,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C2" s="5">
         <v>4017</v>
@@ -1858,7 +1852,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C3">
         <v>1000</v>
@@ -1869,10 +1863,10 @@
         <v>12</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1880,10 +1874,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1891,10 +1885,10 @@
         <v>12</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" t="s">
-        <v>89</v>
+        <v>80</v>
+      </c>
+      <c r="C6">
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1902,10 +1896,10 @@
         <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1913,7 +1907,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C8">
         <v>2000</v>
@@ -1950,7 +1944,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C2" s="5">
         <v>6017</v>
@@ -1961,7 +1955,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C3">
         <v>1000</v>
@@ -1972,10 +1966,10 @@
         <v>12</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1983,10 +1977,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1994,10 +1988,10 @@
         <v>12</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" t="s">
-        <v>89</v>
+        <v>80</v>
+      </c>
+      <c r="C6">
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2005,10 +1999,10 @@
         <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2016,7 +2010,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C8">
         <v>3000</v>
@@ -2052,10 +2046,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2063,10 +2057,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2121,10 +2115,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2179,7 +2173,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -2190,10 +2184,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2201,10 +2195,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2212,10 +2206,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2271,7 +2265,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -2282,7 +2276,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -2293,7 +2287,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -2331,10 +2325,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2390,10 +2384,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2401,7 +2395,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -2412,7 +2406,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -2449,10 +2443,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2460,7 +2454,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -2471,7 +2465,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -2574,10 +2568,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2598,8 +2592,8 @@
       <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
-        <v>22</v>
+      <c r="C10">
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2607,7 +2601,7 @@
         <v>12</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>19</v>
@@ -2644,7 +2638,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -2655,7 +2649,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -2666,7 +2660,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
@@ -2677,7 +2671,7 @@
         <v>12</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s">
         <v>16</v>
@@ -2688,7 +2682,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
         <v>18</v>
@@ -2699,7 +2693,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
@@ -2721,10 +2715,10 @@
         <v>12</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
+        <v>80</v>
+      </c>
+      <c r="C9">
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2732,10 +2726,10 @@
         <v>12</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -2768,10 +2762,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Merged PR 13293: Merge vai_allocation to Temp_Master_Allocation
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\product_automation_allocation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\Product_Auto_Clone\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091B4903-1BC1-45F0-9509-668242BC5C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78DAA2E2-A2BF-407D-BACA-567533A0F303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="5" activeTab="6" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="5" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
@@ -18,28 +18,29 @@
     <sheet name="Subrecipient_SOW_creation" sheetId="17" r:id="rId3"/>
     <sheet name="Budget_Redirection" sheetId="15" r:id="rId4"/>
     <sheet name="Subrecipient_BRedirection" sheetId="21" r:id="rId5"/>
-    <sheet name="Subrecipient_KPC" sheetId="22" r:id="rId6"/>
-    <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId7"/>
-    <sheet name="Subrecipient_SOW_Edition" sheetId="18" r:id="rId8"/>
-    <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId9"/>
-    <sheet name="SubRecipientBPC_Creation" sheetId="19" r:id="rId10"/>
-    <sheet name="Subrecipient_BPCSOW_Creation" sheetId="26" r:id="rId11"/>
-    <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId12"/>
-    <sheet name="SubRecipientBPC_Edition" sheetId="20" r:id="rId13"/>
-    <sheet name="SubRecipientCF_Creation" sheetId="23" r:id="rId14"/>
-    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId15"/>
-    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId16"/>
-    <sheet name="GrantCreation" sheetId="6" r:id="rId17"/>
-    <sheet name="GrantEdition" sheetId="7" r:id="rId18"/>
-    <sheet name="Edition_Standalone" sheetId="8" r:id="rId19"/>
-    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId20"/>
-    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId21"/>
-    <sheet name="Periodic Renewal" sheetId="12" r:id="rId22"/>
-    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId23"/>
-    <sheet name="Periodic Renewal Edition1" sheetId="28" r:id="rId24"/>
-    <sheet name="Funding_Terms_creation" sheetId="24" r:id="rId25"/>
-    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId26"/>
-    <sheet name="AllAmendment_Creation" sheetId="27" r:id="rId27"/>
+    <sheet name="Subrecipient_BRedirec_Carry_Err" sheetId="29" r:id="rId6"/>
+    <sheet name="Subrecipient_KPC" sheetId="22" r:id="rId7"/>
+    <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId8"/>
+    <sheet name="Subrecipient_SOW_Edition" sheetId="18" r:id="rId9"/>
+    <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId10"/>
+    <sheet name="SubRecipientBPC_Creation" sheetId="19" r:id="rId11"/>
+    <sheet name="Subrecipient_BPCSOW_Creation" sheetId="26" r:id="rId12"/>
+    <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId13"/>
+    <sheet name="SubRecipientBPC_Edition" sheetId="20" r:id="rId14"/>
+    <sheet name="SubRecipientCF_Creation" sheetId="23" r:id="rId15"/>
+    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId16"/>
+    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId17"/>
+    <sheet name="GrantCreation" sheetId="6" r:id="rId18"/>
+    <sheet name="GrantEdition" sheetId="7" r:id="rId19"/>
+    <sheet name="Edition_Standalone" sheetId="8" r:id="rId20"/>
+    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId21"/>
+    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId22"/>
+    <sheet name="Periodic Renewal" sheetId="12" r:id="rId23"/>
+    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId24"/>
+    <sheet name="Periodic Renewal Edition1" sheetId="28" r:id="rId25"/>
+    <sheet name="Funding_Terms_creation" sheetId="24" r:id="rId26"/>
+    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId27"/>
+    <sheet name="AllAmendment_Creation" sheetId="27" r:id="rId28"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="97">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -748,7 +749,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -814,6 +815,64 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25797962-2CD8-4222-8F0C-F2737F68CB74}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -872,7 +931,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EBA5DFF-498D-4D83-B948-A4DE3D93557A}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -941,7 +1000,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -989,7 +1048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F116B932-6CC5-49E6-907B-B1FB48B4CADD}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1037,7 +1096,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFB9B001-FDE9-4CB7-8749-6B43410AD625}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1095,7 +1154,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1142,7 +1201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1201,7 +1260,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1314,7 +1373,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1453,53 +1512,6 @@
       </c>
       <c r="C12" t="s">
         <v>39</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C3">
-        <v>3650</v>
       </c>
     </row>
   </sheetData>
@@ -1577,6 +1589,53 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1667,7 +1726,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1758,7 +1817,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF2024B-3855-4F21-818F-72BDEF018EB6}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1816,7 +1875,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6731B0-0A3A-4C99-9219-CD51FBCA919D}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1919,7 +1978,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{553CC38A-2DBF-46D2-8E76-C45CC7EF93DF}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2021,7 +2080,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62770C67-3364-43CF-8FC9-172E7743FC1C}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2090,7 +2149,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01F7F05-2D11-4E6A-A090-87D63AD5B8AF}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2148,7 +2207,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DFDBA76-585A-4956-AF61-28921A0073B1}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2419,6 +2478,75 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2FA7DC5-C4A1-4E9C-B02D-9945A615B758}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F956442-5D32-41A9-9373-4CEFD36ACD4B}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2476,7 +2604,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3C3D45-7E71-472A-AB14-3D5373D782BA}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2612,7 +2740,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B2B8548-7B25-4129-9EB7-BF1BA0DF00C4}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2735,62 +2863,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>